<commit_message>
one last run before handover
</commit_message>
<xml_diff>
--- a/output/table_13_oecd_oda.xlsx
+++ b/output/table_13_oecd_oda.xlsx
@@ -441,7 +441,7 @@
         <v>0.33</v>
       </c>
       <c r="H2">
-        <v>211.869</v>
+        <v>211.874</v>
       </c>
       <c r="I2">
         <v>75.8</v>
@@ -481,7 +481,7 @@
         <v>0.47</v>
       </c>
       <c r="H3">
-        <v>88.34999999999999</v>
+        <v>88.355</v>
       </c>
       <c r="I3">
         <v>62.3</v>
@@ -675,13 +675,13 @@
         <v>-16.6</v>
       </c>
       <c r="F8">
-        <v>-7.4</v>
+        <v>-7.3</v>
       </c>
       <c r="G8">
         <v>0.47</v>
       </c>
       <c r="H8">
-        <v>15.073</v>
+        <v>15.074</v>
       </c>
       <c r="I8">
         <v>55.6</v>
@@ -721,7 +721,7 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="H9">
-        <v>33.245</v>
+        <v>33.249</v>
       </c>
       <c r="I9">
         <v>75.09999999999999</v>
@@ -829,10 +829,10 @@
         <v>6.5</v>
       </c>
       <c r="D12">
-        <v>16.1</v>
+        <v>15.9</v>
       </c>
       <c r="E12">
-        <v>-17.5</v>
+        <v>-17.4</v>
       </c>
       <c r="F12">
         <v>12</v>
@@ -1112,10 +1112,10 @@
         <v>43</v>
       </c>
       <c r="E19">
-        <v>-0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="F19">
-        <v>-8.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="G19">
         <v>0.38</v>

</xml_diff>